<commit_message>
plotting and statistics updated
</commit_message>
<xml_diff>
--- a/plotting_and_statistics_script_with_demo_data/output_files_of_py_script/2024-06-11 02_15_01_statistics_1wire-temperatures.xlsx
+++ b/plotting_and_statistics_script_with_demo_data/output_files_of_py_script/2024-06-11 02_15_01_statistics_1wire-temperatures.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -430,44 +418,44 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Lumar</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>ImagerZ1</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>SZX12_R</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>M165FC</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>SZX12_L</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Axioplan2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>duration [d]</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>count</t>
         </is>
@@ -490,12 +478,12 @@
       <c r="G2" t="n">
         <v>999</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="1" t="n">
         <v>10.39583333333333</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>mean</t>
         </is>
@@ -518,12 +506,12 @@
       <c r="G3" t="n">
         <v>22.34226226226226</v>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="1" t="n">
         <v>10.39583333333333</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>min</t>
         </is>
@@ -546,12 +534,12 @@
       <c r="G4" t="n">
         <v>20.38</v>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="1" t="n">
         <v>10.39583333333333</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -574,12 +562,12 @@
       <c r="G5" t="n">
         <v>21.38</v>
       </c>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="1" t="n">
         <v>10.39583333333333</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>50%</t>
         </is>
@@ -602,12 +590,12 @@
       <c r="G6" t="n">
         <v>22.25</v>
       </c>
-      <c r="H6" s="2" t="n">
+      <c r="H6" s="1" t="n">
         <v>10.39583333333333</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>75%</t>
         </is>
@@ -630,12 +618,12 @@
       <c r="G7" t="n">
         <v>23</v>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="H7" s="1" t="n">
         <v>10.39583333333333</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>max</t>
         </is>
@@ -658,12 +646,12 @@
       <c r="G8" t="n">
         <v>25.94</v>
       </c>
-      <c r="H8" s="2" t="n">
+      <c r="H8" s="1" t="n">
         <v>10.39583333333333</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>std</t>
         </is>
@@ -686,7 +674,7 @@
       <c r="G9" t="n">
         <v>1.217263549271092</v>
       </c>
-      <c r="H9" s="2" t="n">
+      <c r="H9" s="1" t="n">
         <v>10.39583333333333</v>
       </c>
     </row>

</xml_diff>